<commit_message>
modify menu.xls to menu.png
</commit_message>
<xml_diff>
--- a/task/menu.xlsx
+++ b/task/menu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\alantop_dir\alantop_data\alantop_git\github\task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C35F07A-C8E6-4E16-8185-E19677C6CF35}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA7533E-73EF-48CF-A1F7-37CD4D24DA61}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -489,8 +489,7 @@
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="38" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.44140625" style="1" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
modify menu and zhang bill
</commit_message>
<xml_diff>
--- a/task/menu.xlsx
+++ b/task/menu.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\alantop_dir\alantop_data\alantop_git\github\task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA7533E-73EF-48CF-A1F7-37CD4D24DA61}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3BF82B-0BC9-4F73-B79F-521115CDE181}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="32">
   <si>
     <t>星期一</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -71,10 +72,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>牛排，</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>胡椒猪肚鸡汤米线</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -87,19 +84,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>冬菇滑鸡粥，</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>韩式海鲜辛拉面，</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>猪肝粥，</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>净云吞，</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -136,6 +121,42 @@
     <t>优火锅
  （日式清汤，乌冬，
 牛肉，冻柠檬茶）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>咖喱牛腩</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>黑胡椒鸡排</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>subway</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>净云吞</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>牛排</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>彪记 手撕鸡</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>胡椒猪肚鸡米线</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>subway</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>猪肝粥</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -143,7 +164,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,6 +174,32 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
@@ -194,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -204,6 +251,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -485,11 +547,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr defaultRowHeight="22.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="3" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -498,143 +561,258 @@
     <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="6"/>
+      <c r="B1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCAF2C29-90A3-40D0-8A09-AB67368DA2F7}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="82.8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="69" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="82.8" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="69" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="B6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="B7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="41.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="1" t="s">
-        <v>23</v>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>